<commit_message>
Validación de objetivos primera etapa
</commit_message>
<xml_diff>
--- a/PlantillaMVC/Export/Temp3.xlsx
+++ b/PlantillaMVC/Export/Temp3.xlsx
@@ -14,7 +14,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<x:sst xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="25" uniqueCount="25">
+<x:sst xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="11" uniqueCount="11">
   <x:si>
     <x:t>Numero Empleado SAP</x:t>
   </x:si>
@@ -40,55 +40,13 @@
     <x:t>Métrica</x:t>
   </x:si>
   <x:si>
-    <x:t>Peso del objetivo(%)</x:t>
-  </x:si>
-  <x:si>
     <x:t>Resultado</x:t>
   </x:si>
   <x:si>
     <x:t>Comentarios jefe</x:t>
   </x:si>
   <x:si>
-    <x:t xml:space="preserve">Vacante Vac </x:t>
-  </x:si>
-  <x:si>
-    <x:t>Vacante</x:t>
-  </x:si>
-  <x:si>
-    <x:t>Felipe Vargas Vargas</x:t>
-  </x:si>
-  <x:si>
-    <x:t>Sin objetivos en el periodo</x:t>
-  </x:si>
-  <x:si>
-    <x:t>Hector Rodrigo Vargas Vargas</x:t>
-  </x:si>
-  <x:si>
-    <x:t>Tester</x:t>
-  </x:si>
-  <x:si>
-    <x:t>a</x:t>
-  </x:si>
-  <x:si>
-    <x:t>solo el 92%</x:t>
-  </x:si>
-  <x:si>
-    <x:t>queda a un 95%</x:t>
-  </x:si>
-  <x:si>
-    <x:t>b</x:t>
-  </x:si>
-  <x:si>
-    <x:t>se cumple al 100%</x:t>
-  </x:si>
-  <x:si>
-    <x:t>c</x:t>
-  </x:si>
-  <x:si>
-    <x:t>completado al 100%</x:t>
-  </x:si>
-  <x:si>
-    <x:t>queda a un 90%</x:t>
+    <x:t>Peso ponderado %</x:t>
   </x:si>
 </x:sst>
 </file>
@@ -115,7 +73,7 @@
       <x:family val="2"/>
     </x:font>
   </x:fonts>
-  <x:fills count="4">
+  <x:fills count="3">
     <x:fill>
       <x:patternFill patternType="none"/>
     </x:fill>
@@ -126,12 +84,6 @@
       <x:patternFill patternType="solid">
         <x:fgColor rgb="FFF0F8FF"/>
         <x:bgColor rgb="FFF0F8FF"/>
-      </x:patternFill>
-    </x:fill>
-    <x:fill>
-      <x:patternFill patternType="solid">
-        <x:fgColor rgb="FFFFFFE0"/>
-        <x:bgColor rgb="FFFFFFE0"/>
       </x:patternFill>
     </x:fill>
   </x:fills>
@@ -154,7 +106,7 @@
       </x:diagonal>
     </x:border>
   </x:borders>
-  <x:cellStyleXfs count="8">
+  <x:cellStyleXfs count="4">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyNumberFormat="0" applyFill="1" applyBorder="0" applyAlignment="0" applyProtection="1">
       <x:protection locked="1" hidden="0"/>
     </x:xf>
@@ -164,23 +116,11 @@
     <x:xf numFmtId="0" fontId="1" fillId="2" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="1">
       <x:protection locked="1" hidden="0"/>
     </x:xf>
-    <x:xf numFmtId="0" fontId="0" fillId="3" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="1">
-      <x:protection locked="1" hidden="0"/>
-    </x:xf>
-    <x:xf numFmtId="0" fontId="0" fillId="3" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="1">
-      <x:protection locked="1" hidden="0"/>
-    </x:xf>
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyNumberFormat="0" applyFill="1" applyBorder="0" applyAlignment="0" applyProtection="1">
       <x:protection locked="1" hidden="0"/>
     </x:xf>
-    <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyNumberFormat="0" applyFill="1" applyBorder="0" applyAlignment="0" applyProtection="1">
-      <x:protection locked="1" hidden="0"/>
-    </x:xf>
-    <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyNumberFormat="0" applyFill="1" applyBorder="0" applyAlignment="0" applyProtection="1">
-      <x:protection locked="1" hidden="0"/>
-    </x:xf>
   </x:cellStyleXfs>
-  <x:cellXfs count="8">
+  <x:cellXfs count="4">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="0" applyFill="1" applyBorder="0" applyAlignment="0" applyProtection="1">
       <x:alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="0" indent="0" relativeIndent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
       <x:protection locked="1" hidden="0"/>
@@ -191,22 +131,6 @@
     </x:xf>
     <x:xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="1">
       <x:alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="1" indent="0" relativeIndent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-      <x:protection locked="1" hidden="0"/>
-    </x:xf>
-    <x:xf numFmtId="0" fontId="0" fillId="3" borderId="0" xfId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="1">
-      <x:alignment horizontal="general" vertical="center" textRotation="0" wrapText="0" indent="0" relativeIndent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-      <x:protection locked="1" hidden="0"/>
-    </x:xf>
-    <x:xf numFmtId="0" fontId="0" fillId="3" borderId="0" xfId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="1">
-      <x:alignment horizontal="general" vertical="center" textRotation="0" wrapText="1" indent="0" relativeIndent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-      <x:protection locked="1" hidden="0"/>
-    </x:xf>
-    <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="0" applyFill="1" applyBorder="0" applyAlignment="0" applyProtection="1">
-      <x:alignment horizontal="general" vertical="center" textRotation="0" wrapText="0" indent="0" relativeIndent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-      <x:protection locked="1" hidden="0"/>
-    </x:xf>
-    <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="0" applyFill="1" applyBorder="0" applyAlignment="0" applyProtection="1">
-      <x:alignment horizontal="general" vertical="center" textRotation="0" wrapText="1" indent="0" relativeIndent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
       <x:protection locked="1" hidden="0"/>
     </x:xf>
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="0" applyFill="1" applyBorder="0" applyAlignment="0" applyProtection="1">
@@ -508,14 +432,14 @@
   <x:sheetPr>
     <x:outlinePr summaryBelow="1" summaryRight="1"/>
   </x:sheetPr>
-  <x:dimension ref="A1:K5"/>
+  <x:dimension ref="A1:K1"/>
   <x:sheetFormatPr defaultRowHeight="15"/>
   <x:cols>
     <x:col min="1" max="1" width="15.710625" style="0" customWidth="1"/>
     <x:col min="2" max="4" width="35.710625" style="0" customWidth="1"/>
     <x:col min="5" max="6" width="40.710625" style="0" customWidth="1"/>
-    <x:col min="7" max="7" width="40.710625" style="7" customWidth="1"/>
-    <x:col min="8" max="8" width="45.710625" style="7" customWidth="1"/>
+    <x:col min="7" max="7" width="40.710625" style="3" customWidth="1"/>
+    <x:col min="8" max="8" width="45.710625" style="3" customWidth="1"/>
     <x:col min="9" max="11" width="45.710625" style="0" customWidth="1"/>
   </x:cols>
   <x:sheetData>
@@ -552,136 +476,6 @@
       </x:c>
       <x:c r="K1" s="1" t="s">
         <x:v>10</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="2" spans="1:11" s="3" customFormat="1">
-      <x:c r="A2" s="3" t="n">
-        <x:v>1</x:v>
-      </x:c>
-      <x:c r="B2" s="3" t="s">
-        <x:v>11</x:v>
-      </x:c>
-      <x:c r="C2" s="3" t="n">
-        <x:v>1</x:v>
-      </x:c>
-      <x:c r="D2" s="3" t="s">
-        <x:v>12</x:v>
-      </x:c>
-      <x:c r="E2" s="3" t="s">
-        <x:v>13</x:v>
-      </x:c>
-      <x:c r="F2" s="3" t="s">
-        <x:v>14</x:v>
-      </x:c>
-      <x:c r="G2" s="4" t="s"/>
-      <x:c r="H2" s="4" t="s"/>
-      <x:c r="I2" s="3" t="s"/>
-      <x:c r="J2" s="3" t="s"/>
-      <x:c r="K2" s="3" t="s"/>
-    </x:row>
-    <x:row r="3" spans="1:11" s="5" customFormat="1">
-      <x:c r="A3" s="5" t="n">
-        <x:v>15072017</x:v>
-      </x:c>
-      <x:c r="B3" s="5" t="s">
-        <x:v>15</x:v>
-      </x:c>
-      <x:c r="C3" s="5" t="n">
-        <x:v>1</x:v>
-      </x:c>
-      <x:c r="D3" s="5" t="s">
-        <x:v>16</x:v>
-      </x:c>
-      <x:c r="E3" s="5" t="s">
-        <x:v>13</x:v>
-      </x:c>
-      <x:c r="F3" s="5" t="s">
-        <x:v>17</x:v>
-      </x:c>
-      <x:c r="G3" s="6" t="s">
-        <x:v>17</x:v>
-      </x:c>
-      <x:c r="H3" s="6" t="s">
-        <x:v>17</x:v>
-      </x:c>
-      <x:c r="I3" s="5" t="n">
-        <x:v>50</x:v>
-      </x:c>
-      <x:c r="J3" s="5" t="s">
-        <x:v>18</x:v>
-      </x:c>
-      <x:c r="K3" s="5" t="s">
-        <x:v>19</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="4" spans="1:11" s="5" customFormat="1">
-      <x:c r="A4" s="5" t="n">
-        <x:v>15072017</x:v>
-      </x:c>
-      <x:c r="B4" s="5" t="s">
-        <x:v>15</x:v>
-      </x:c>
-      <x:c r="C4" s="5" t="n">
-        <x:v>1</x:v>
-      </x:c>
-      <x:c r="D4" s="5" t="s">
-        <x:v>16</x:v>
-      </x:c>
-      <x:c r="E4" s="5" t="s">
-        <x:v>13</x:v>
-      </x:c>
-      <x:c r="F4" s="5" t="s">
-        <x:v>20</x:v>
-      </x:c>
-      <x:c r="G4" s="6" t="s">
-        <x:v>20</x:v>
-      </x:c>
-      <x:c r="H4" s="6" t="s">
-        <x:v>20</x:v>
-      </x:c>
-      <x:c r="I4" s="5" t="n">
-        <x:v>30</x:v>
-      </x:c>
-      <x:c r="J4" s="5" t="s">
-        <x:v>21</x:v>
-      </x:c>
-      <x:c r="K4" s="5" t="s">
-        <x:v>21</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="5" spans="1:11">
-      <x:c r="A5" s="0" t="n">
-        <x:v>15072017</x:v>
-      </x:c>
-      <x:c r="B5" s="0" t="s">
-        <x:v>15</x:v>
-      </x:c>
-      <x:c r="C5" s="0" t="n">
-        <x:v>1</x:v>
-      </x:c>
-      <x:c r="D5" s="0" t="s">
-        <x:v>16</x:v>
-      </x:c>
-      <x:c r="E5" s="0" t="s">
-        <x:v>13</x:v>
-      </x:c>
-      <x:c r="F5" s="0" t="s">
-        <x:v>22</x:v>
-      </x:c>
-      <x:c r="G5" s="7" t="s">
-        <x:v>22</x:v>
-      </x:c>
-      <x:c r="H5" s="7" t="s">
-        <x:v>22</x:v>
-      </x:c>
-      <x:c r="I5" s="0" t="n">
-        <x:v>20</x:v>
-      </x:c>
-      <x:c r="J5" s="0" t="s">
-        <x:v>23</x:v>
-      </x:c>
-      <x:c r="K5" s="0" t="s">
-        <x:v>24</x:v>
       </x:c>
     </x:row>
   </x:sheetData>

</xml_diff>